<commit_message>
Update project and .gitignore for Demo branch
</commit_message>
<xml_diff>
--- a/data_files/brokerage_fact/FY746(Feb 26 brkg).xlsx
+++ b/data_files/brokerage_fact/FY746(Feb 26 brkg).xlsx
@@ -1,12 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\SalesDashboardProject (2) (1)\SalesDashboardProject\data_files\brokerage_fact\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4545"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -130,25 +138,25 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -158,7 +166,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -168,37 +176,40 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -206,7 +217,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -396,17 +407,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AA18"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="18" max="18" width="36.7109375" customWidth="1"/>
+    <col min="19" max="19" width="37.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,7 +507,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -497,82 +515,82 @@
         <v>28</v>
       </c>
       <c r="C2" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D2" s="4">
         <v>566.75</v>
       </c>
       <c r="E2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F2" s="4">
         <v>566.75</v>
       </c>
       <c r="G2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L2" s="4">
-        <v>113350.0</v>
+        <v>113350</v>
       </c>
       <c r="M2" s="4">
-        <v>113350.0</v>
+        <v>113350</v>
       </c>
       <c r="N2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="4">
-        <v>113350.0</v>
+        <v>113350</v>
       </c>
       <c r="R2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T2" s="4">
-        <v>113350.0</v>
+        <v>113350</v>
       </c>
       <c r="U2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z2" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA2" s="4">
         <v>566.75</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -580,7 +598,7 @@
         <v>28</v>
       </c>
       <c r="C3" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D3" s="4">
         <v>450.04</v>
@@ -592,16 +610,16 @@
         <v>452.44</v>
       </c>
       <c r="G3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K3" s="4">
         <v>9607.1</v>
@@ -613,49 +631,49 @@
         <v>189092.6</v>
       </c>
       <c r="N3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="4">
         <v>189092.6</v>
       </c>
       <c r="R3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T3" s="4">
         <v>189092.6</v>
       </c>
       <c r="U3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA3" s="4">
         <v>452.44</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
@@ -663,31 +681,31 @@
         <v>28</v>
       </c>
       <c r="C4" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D4" s="4">
         <v>154.49</v>
       </c>
       <c r="E4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F4" s="4">
         <v>154.49</v>
       </c>
       <c r="G4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L4" s="4">
         <v>56805.14</v>
@@ -696,81 +714,81 @@
         <v>56805.14</v>
       </c>
       <c r="N4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="4">
         <v>56805.14</v>
       </c>
       <c r="R4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T4" s="4">
         <v>56805.14</v>
       </c>
       <c r="U4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="4">
         <v>154.49</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
-        <v>9.8307865E7</v>
+        <v>98307865</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D5" s="4">
         <v>106.83</v>
       </c>
       <c r="E5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F5" s="4">
         <v>106.83</v>
       </c>
       <c r="G5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L5" s="4">
         <v>42731.5</v>
@@ -779,49 +797,49 @@
         <v>42731.5</v>
       </c>
       <c r="N5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="4">
         <v>42731.5</v>
       </c>
       <c r="R5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T5" s="4">
         <v>42731.5</v>
       </c>
       <c r="U5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="4">
         <v>106.83</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -829,31 +847,31 @@
         <v>28</v>
       </c>
       <c r="C6" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D6" s="4">
         <v>31.05</v>
       </c>
       <c r="E6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F6" s="4">
         <v>31.05</v>
       </c>
       <c r="G6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L6" s="4">
         <v>6209.9</v>
@@ -862,49 +880,49 @@
         <v>6209.9</v>
       </c>
       <c r="N6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="4">
         <v>6209.9</v>
       </c>
       <c r="R6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T6" s="4">
         <v>6209.9</v>
       </c>
       <c r="U6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="4">
         <v>31.05</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
@@ -912,40 +930,40 @@
         <v>28</v>
       </c>
       <c r="C7" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="I7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O7" s="4">
         <v>185997.3</v>
@@ -957,37 +975,37 @@
         <v>185997.3</v>
       </c>
       <c r="R7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T7" s="4">
         <v>185997.3</v>
       </c>
       <c r="U7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="4">
-        <v>100.0</v>
+        <v>100</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
@@ -995,82 +1013,82 @@
         <v>28</v>
       </c>
       <c r="C8" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4">
         <v>1340.93</v>
       </c>
       <c r="H8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N8" s="4">
-        <v>2681850.0</v>
+        <v>2681850</v>
       </c>
       <c r="O8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P8" s="4">
-        <v>2681850.0</v>
+        <v>2681850</v>
       </c>
       <c r="Q8" s="4">
-        <v>2681850.0</v>
+        <v>2681850</v>
       </c>
       <c r="R8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T8" s="4">
-        <v>2681850.0</v>
+        <v>2681850</v>
       </c>
       <c r="U8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="4">
         <v>1340.93</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
@@ -1078,40 +1096,40 @@
         <v>28</v>
       </c>
       <c r="C9" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H9" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O9" s="4">
         <v>1240.5</v>
@@ -1123,37 +1141,37 @@
         <v>1240.5</v>
       </c>
       <c r="R9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T9" s="4">
         <v>1240.5</v>
       </c>
       <c r="U9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA9" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
@@ -1161,82 +1179,82 @@
         <v>28</v>
       </c>
       <c r="C10" s="3">
-        <v>46054.0</v>
+        <v>46054</v>
       </c>
       <c r="D10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4">
         <v>2400.02</v>
       </c>
       <c r="I10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O10" s="4">
-        <v>420560.0</v>
+        <v>420560</v>
       </c>
       <c r="P10" s="4">
-        <v>420560.0</v>
+        <v>420560</v>
       </c>
       <c r="Q10" s="4">
-        <v>420560.0</v>
+        <v>420560</v>
       </c>
       <c r="R10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T10" s="4">
-        <v>420560.0</v>
+        <v>420560</v>
       </c>
       <c r="U10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="4">
         <v>2400.02</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
@@ -1244,31 +1262,31 @@
         <v>28</v>
       </c>
       <c r="C11" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D11" s="4">
-        <v>4893.85</v>
+        <v>4893.8500000000004</v>
       </c>
       <c r="E11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F11" s="4">
-        <v>4893.85</v>
+        <v>4893.8500000000004</v>
       </c>
       <c r="G11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L11" s="4">
         <v>978770.5</v>
@@ -1277,49 +1295,49 @@
         <v>978770.5</v>
       </c>
       <c r="N11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="4">
         <v>978770.5</v>
       </c>
       <c r="R11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T11" s="4">
         <v>978770.5</v>
       </c>
       <c r="U11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="4">
-        <v>4893.85</v>
+        <v>4893.8500000000004</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
@@ -1327,13 +1345,13 @@
         <v>28</v>
       </c>
       <c r="C12" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D12" s="4">
         <v>342.01</v>
       </c>
       <c r="E12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F12" s="4">
         <v>342.01</v>
@@ -1342,16 +1360,16 @@
         <v>327.49</v>
       </c>
       <c r="H12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L12" s="4">
         <v>68402.8</v>
@@ -1363,7 +1381,7 @@
         <v>654977.5</v>
       </c>
       <c r="O12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P12" s="4">
         <v>654977.5</v>
@@ -1372,37 +1390,37 @@
         <v>723380.3</v>
       </c>
       <c r="R12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T12" s="4">
         <v>723380.3</v>
       </c>
       <c r="U12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="4">
         <v>669.5</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -1410,7 +1428,7 @@
         <v>28</v>
       </c>
       <c r="C13" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D13" s="4">
         <v>131.74</v>
@@ -1422,19 +1440,19 @@
         <v>135.07</v>
       </c>
       <c r="G13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K13" s="4">
-        <v>13300.0</v>
+        <v>13300</v>
       </c>
       <c r="L13" s="4">
         <v>48818.97</v>
@@ -1443,49 +1461,49 @@
         <v>62118.97</v>
       </c>
       <c r="N13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="4">
         <v>62118.97</v>
       </c>
       <c r="R13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T13" s="4">
         <v>62118.97</v>
       </c>
       <c r="U13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="4">
         <v>135.07</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:27" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -1493,31 +1511,31 @@
         <v>28</v>
       </c>
       <c r="C14" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D14" s="4">
         <v>86.3</v>
       </c>
       <c r="E14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F14" s="4">
         <v>86.3</v>
       </c>
       <c r="G14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L14" s="4">
         <v>29086.5</v>
@@ -1526,49 +1544,49 @@
         <v>29086.5</v>
       </c>
       <c r="N14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="4">
         <v>29086.5</v>
       </c>
       <c r="R14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T14" s="4">
         <v>29086.5</v>
       </c>
       <c r="U14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="4">
         <v>86.3</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:27" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>31</v>
       </c>
@@ -1576,31 +1594,31 @@
         <v>28</v>
       </c>
       <c r="C15" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D15" s="4">
         <v>46.4</v>
       </c>
       <c r="E15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F15" s="4">
         <v>46.4</v>
       </c>
       <c r="G15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L15" s="4">
         <v>9279.5</v>
@@ -1609,49 +1627,49 @@
         <v>9279.5</v>
       </c>
       <c r="N15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="4">
         <v>9279.5</v>
       </c>
       <c r="R15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T15" s="4">
         <v>9279.5</v>
       </c>
       <c r="U15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z15" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA15" s="4">
         <v>46.4</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:27" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>37</v>
       </c>
@@ -1659,31 +1677,31 @@
         <v>28</v>
       </c>
       <c r="C16" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D16" s="4">
         <v>0.11</v>
       </c>
       <c r="E16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F16" s="4">
         <v>0.11</v>
       </c>
       <c r="G16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L16" s="4">
         <v>10999.89</v>
@@ -1692,49 +1710,49 @@
         <v>10999.89</v>
       </c>
       <c r="N16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="P16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="4">
         <v>10999.89</v>
       </c>
       <c r="R16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T16" s="4">
         <v>10999.89</v>
       </c>
       <c r="U16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z16" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA16" s="4">
         <v>0.11</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:27" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -1742,40 +1760,40 @@
         <v>28</v>
       </c>
       <c r="C17" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="I17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O17" s="4">
         <v>1382.5</v>
@@ -1787,37 +1805,37 @@
         <v>1382.5</v>
       </c>
       <c r="R17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T17" s="4">
         <v>1382.5</v>
       </c>
       <c r="U17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z17" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA17" s="4">
-        <v>15.0</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:27" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -1825,40 +1843,40 @@
         <v>28</v>
       </c>
       <c r="C18" s="3">
-        <v>46055.0</v>
+        <v>46055</v>
       </c>
       <c r="D18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="I18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="J18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="K18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="O18" s="4">
         <v>93042.5</v>
@@ -1870,37 +1888,37 @@
         <v>93042.5</v>
       </c>
       <c r="R18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="S18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T18" s="4">
         <v>93042.5</v>
       </c>
       <c r="U18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="V18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="W18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="X18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="4">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="4">
-        <v>50.0</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>